<commit_message>
fixed marked_514 0813 recording
</commit_message>
<xml_diff>
--- a/Vocalization_recording_data.xlsx
+++ b/Vocalization_recording_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2a96053f85c76562/Documents/GitHub/Vocalizations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="62" documentId="13_ncr:1_{22C56AFF-B3E7-4B78-9FD8-38F58A352E93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17CCD501-8C47-4553-A71C-B8A76BF4C01D}"/>
+  <xr:revisionPtr revIDLastSave="63" documentId="13_ncr:1_{22C56AFF-B3E7-4B78-9FD8-38F58A352E93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6B66C37E-435F-4BAB-8B34-3802AA25812D}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{A86565EC-7D4E-FF45-BCFA-45F936026A54}"/>
+    <workbookView minimized="1" xWindow="3190" yWindow="2660" windowWidth="14400" windowHeight="8170" xr2:uid="{A86565EC-7D4E-FF45-BCFA-45F936026A54}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -487,7 +487,7 @@
     <col min="4" max="4" width="29.08203125" customWidth="1"/>
     <col min="5" max="7" width="16" customWidth="1"/>
     <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="28.1640625" customWidth="1"/>
+    <col min="9" max="9" width="35.75" customWidth="1"/>
     <col min="10" max="10" width="14.08203125" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
fixed recording name formatting, added note to anesthesia-only control
</commit_message>
<xml_diff>
--- a/Vocalization_recording_data.xlsx
+++ b/Vocalization_recording_data.xlsx
@@ -1,42 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2a96053f85c76562/Documents/GitHub/Vocalizations/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/omer/Desktop/Vocalizations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="154" documentId="13_ncr:1_{22C56AFF-B3E7-4B78-9FD8-38F58A352E93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F8544B6D-455D-47B1-829A-143205DE52CF}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72188A45-025D-3A4E-8D88-476D623C5518}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{A86565EC-7D4E-FF45-BCFA-45F936026A54}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="19420" windowHeight="11500" xr2:uid="{A86565EC-7D4E-FF45-BCFA-45F936026A54}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t>CAGE NUMBER</t>
   </si>
@@ -134,34 +123,37 @@
     <t>Gain2</t>
   </si>
   <si>
-    <t>marked_867352_260918</t>
-  </si>
-  <si>
-    <t>marked_870595_260918</t>
-  </si>
-  <si>
-    <t>unmarked_867352_260918</t>
-  </si>
-  <si>
-    <t>unmarked_870595_260918</t>
-  </si>
-  <si>
-    <t>marked_867352_261009</t>
-  </si>
-  <si>
-    <t>unmarked_867352_261009</t>
-  </si>
-  <si>
-    <t>marked_870595_261009</t>
-  </si>
-  <si>
-    <t>unmarked_870595_261009</t>
-  </si>
-  <si>
     <t>Notes</t>
   </si>
   <si>
     <t>Poor scar.</t>
+  </si>
+  <si>
+    <t>marked_867352_261009.wav</t>
+  </si>
+  <si>
+    <t>unmarked_867352_261009.wav</t>
+  </si>
+  <si>
+    <t>marked_870595_261009.wav</t>
+  </si>
+  <si>
+    <t>unmarked_870595_261009.wav</t>
+  </si>
+  <si>
+    <t>marked_867352_260918.wav</t>
+  </si>
+  <si>
+    <t>unmarked_867352_260918.wav</t>
+  </si>
+  <si>
+    <t>marked_870595_260918.wav</t>
+  </si>
+  <si>
+    <t>unmarked_870595_260918.wav</t>
+  </si>
+  <si>
+    <t>Anesthesia only.</t>
   </si>
 </sst>
 </file>
@@ -233,9 +225,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -273,7 +265,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -379,7 +371,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -521,7 +513,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -530,18 +522,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90440726-6508-7B45-9053-6C2454E26D68}">
   <dimension ref="A1:M18"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="29.08203125" customWidth="1"/>
-    <col min="5" max="5" width="10.58203125" customWidth="1"/>
+    <col min="4" max="4" width="29" customWidth="1"/>
+    <col min="5" max="5" width="10.5" customWidth="1"/>
     <col min="6" max="8" width="16" customWidth="1"/>
     <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="35.75" customWidth="1"/>
-    <col min="11" max="11" width="9.4140625" customWidth="1"/>
-    <col min="12" max="12" width="14.08203125" customWidth="1"/>
+    <col min="10" max="10" width="35.6640625" customWidth="1"/>
+    <col min="11" max="11" width="9.33203125" customWidth="1"/>
+    <col min="12" max="12" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -579,10 +571,10 @@
         <v>6</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
         <v>853626</v>
       </c>
@@ -618,7 +610,7 @@
       </c>
       <c r="L2" s="2"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>853626</v>
       </c>
@@ -654,7 +646,7 @@
       </c>
       <c r="L3" s="2"/>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>857516</v>
       </c>
@@ -689,7 +681,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>857516</v>
       </c>
@@ -724,7 +716,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>857515</v>
       </c>
@@ -759,7 +751,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>857515</v>
       </c>
@@ -794,7 +786,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>857514</v>
       </c>
@@ -829,7 +821,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>857514</v>
       </c>
@@ -864,7 +856,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>857513</v>
       </c>
@@ -899,7 +891,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>857513</v>
       </c>
@@ -934,7 +926,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>867352</v>
       </c>
@@ -945,7 +937,7 @@
         <v>23</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="E12" s="2">
         <v>10</v>
@@ -964,13 +956,13 @@
         <v>26</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="K12" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>867352</v>
       </c>
@@ -981,7 +973,7 @@
         <v>23</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="E13" s="2">
         <v>10</v>
@@ -999,13 +991,13 @@
         <v>26</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K13" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>870595</v>
       </c>
@@ -1016,7 +1008,7 @@
         <v>15</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="E14" s="2">
         <v>10</v>
@@ -1034,13 +1026,16 @@
         <v>18</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="K14" s="2">
         <v>6</v>
       </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="M14" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>870595</v>
       </c>
@@ -1051,7 +1046,7 @@
         <v>15</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="E15" s="2">
         <v>10</v>
@@ -1069,20 +1064,20 @@
         <v>18</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="K15" s="2">
         <v>6</v>
       </c>
       <c r="M15" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="17" spans="6:7" x14ac:dyDescent="0.35">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="6:7" x14ac:dyDescent="0.2">
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="6:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="6:7" x14ac:dyDescent="0.2">
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
     </row>

</xml_diff>